<commit_message>
feat: Fix search textboxes in reconciliation tabs, fix double-handler RowNotInTableException in suggestion grid, fix row deletion crash in Sanad2Form
- Add SetupSearchForGrid call in SetupSuggestionGridButtonsAndColors so search textboxes appear in suggestion tabs
- Improve ApplyGridFilter to support DataTable/BindingSource and handle Persian column names with parentheses
- Fix tcMain.SelectedIndexChanged to also align grids in nested tcBank/tcAsnad tabs
- Remove dgvAsnad_Suggestions from dgvAsnad_CellContentClick Handles to prevent double-fire RowNotInTableException
- Merge btnEditSanadCol and btnResolveCol logic into single dgvSuggestions_CellContentClick handler with safe row access
- Fix RowNotInTableException in HesabdarySanad2Form DgvEntryLines_SelectionChanged by checking DataRowState.Deleted
- Fix RenumberRows to skip deleted rows and renumber correctly
- Wrap UpdateRowInfoLabels in try-catch to prevent crash after row removal
</commit_message>
<xml_diff>
--- a/sath_dastresy.xlsx
+++ b/sath_dastresy.xlsx
@@ -9,11 +9,16 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="5895" windowHeight="5835"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="5895" windowHeight="5835" firstSheet="4" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="مرتب بر اساس ستون مجوز" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet4" sheetId="5" r:id="rId3"/>
+    <sheet name="مشارکتی گروه B" sheetId="4" r:id="rId4"/>
+    <sheet name="جدول شماره 8 - مشارکتی گروه B" sheetId="6" r:id="rId5"/>
+    <sheet name="جدول شماره 9 - مشارکتی گ B" sheetId="7" r:id="rId6"/>
+    <sheet name="جدول سود وزیان-انفرادی گروه B" sheetId="8" r:id="rId7"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="125">
   <si>
     <t>تنظیمات سیستم</t>
   </si>
@@ -235,6 +240,171 @@
   </si>
   <si>
     <t>022</t>
+  </si>
+  <si>
+    <t>جدول شماره :٣خلاصه فھرست درآمدھای حاصل از شراکت</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ردیف </t>
+  </si>
+  <si>
+    <t>شرح</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> مبلغ</t>
+  </si>
+  <si>
+    <t>سود (زیان) ویژه (نقل از جدول ٨)</t>
+  </si>
+  <si>
+    <t>اضافھ/ کسر میشود از سود (زیان) خالص</t>
+  </si>
+  <si>
+    <t>اضافه/ کسر میشود از سود (زیان) خالص</t>
+  </si>
+  <si>
+    <t>سود حاصل از درآمدھایی کھ مالیات آن قبلاً بھ طور مقطوع پرداخت شده (نقل از جدول ٧)</t>
+  </si>
+  <si>
+    <t>درآمدھای معاف (نقل از جدول ۴)</t>
+  </si>
+  <si>
+    <t>جمع تعدیلات =(٣+۴)-٢</t>
+  </si>
+  <si>
+    <t>درآمد مشمول مالیات قبل از کسر معافیت ماده ١٠١ قمم (زیان سال جاری)</t>
+  </si>
+  <si>
+    <t>جدول :۱-٣ محاسبه درآمد مشمول مالیات قبل از کسر معافیت ماده ١٠١ ق م م</t>
+  </si>
+  <si>
+    <t>جدول شماره :٨ صورت درآمد و ھزینه و محاسبه سود و زیان ویژه</t>
+  </si>
+  <si>
+    <t>از تاریخ /..../.... ........</t>
+  </si>
+  <si>
+    <t>تا تاریخ /..../.... ........</t>
+  </si>
+  <si>
+    <t>ردیف</t>
+  </si>
+  <si>
+    <t>سال جاری</t>
+  </si>
+  <si>
+    <t>سال قبل</t>
+  </si>
+  <si>
+    <t>فروش کالا</t>
+  </si>
+  <si>
+    <t>درآمد حاصل از ارائھ خدمات</t>
+  </si>
+  <si>
+    <t>درآمد حاصل از فروش داراییھا</t>
+  </si>
+  <si>
+    <t>سایر درآمدھا</t>
+  </si>
+  <si>
+    <t>جمع فروش و درآمدھا</t>
+  </si>
+  <si>
+    <t>خرید کال</t>
+  </si>
+  <si>
+    <t>جمع خرید و هزینه ها</t>
+  </si>
+  <si>
+    <t>کسرمی شود:موجودی اول دوره</t>
+  </si>
+  <si>
+    <t>سود(زیان) ویژه</t>
+  </si>
+  <si>
+    <t>اضافه می شود:موجودی پایان دوره</t>
+  </si>
+  <si>
+    <t>سایر ھزینه ھا</t>
+  </si>
+  <si>
+    <t>هزینه اجاره محل</t>
+  </si>
+  <si>
+    <t>هزینه حقوق و دستمزد</t>
+  </si>
+  <si>
+    <t>هزینه استھلاک داراییھا</t>
+  </si>
+  <si>
+    <t>هزینه آب، برق، گاز، تلفن</t>
+  </si>
+  <si>
+    <t>جدول شماره :٩ موجودی مواد و کال</t>
+  </si>
+  <si>
+    <t>شرح حساب</t>
+  </si>
+  <si>
+    <t>بهای تمام شده در ابتدای دوره</t>
+  </si>
+  <si>
+    <t>خرید / تولید طی دوره</t>
+  </si>
+  <si>
+    <t>فروش / مصرف طی دوره</t>
+  </si>
+  <si>
+    <t>بهای تمام شده در پایان دوره</t>
+  </si>
+  <si>
+    <t>موجودی سال قبل</t>
+  </si>
+  <si>
+    <t>کالای ساختھ شده</t>
+  </si>
+  <si>
+    <t>کالای در جریان ساخت</t>
+  </si>
+  <si>
+    <t>مواد اولیھ مستقیم</t>
+  </si>
+  <si>
+    <t>مواد کمکی و بستھ بندی</t>
+  </si>
+  <si>
+    <t>قطعات و لوازم یدکی</t>
+  </si>
+  <si>
+    <t>کالای امانی نزد دیگران</t>
+  </si>
+  <si>
+    <t>سایر موجودیھا</t>
+  </si>
+  <si>
+    <t>مواد و کالای در راه</t>
+  </si>
+  <si>
+    <t>بخش ب- محاسبه مالیات</t>
+  </si>
+  <si>
+    <t>مبلغ</t>
+  </si>
+  <si>
+    <t>سود (زیان) ویژه (نقل از جدول ٧</t>
+  </si>
+  <si>
+    <t>سود حاصل از درآمدھایی کھ مالیات آن قبلاً بھ طور مقطوع پرداخت شده (نقل از جدول ۶</t>
+  </si>
+  <si>
+    <t>درآمدھای معاف و موارد قابل کسر از درآمد مشمول مالیات (نقل از جدول ٣</t>
+  </si>
+  <si>
+    <t>کمکھای پرداختی(نقل از جدول ۴</t>
+  </si>
+  <si>
+    <t>جمع تعدیلات     (4 + 5 + 3 ) - 2 =</t>
   </si>
 </sst>
 </file>
@@ -250,12 +420,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -270,7 +446,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -285,6 +461,10 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1656,4 +1836,366 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="H2:J11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="7" max="7" width="9.28515625" customWidth="1"/>
+    <col min="8" max="8" width="14.85546875" customWidth="1"/>
+    <col min="9" max="9" width="65.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="8:10" x14ac:dyDescent="0.25">
+      <c r="J2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="3" spans="8:10" x14ac:dyDescent="0.25">
+      <c r="J3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="5" spans="8:10" x14ac:dyDescent="0.25">
+      <c r="H5" t="s">
+        <v>73</v>
+      </c>
+      <c r="I5" t="s">
+        <v>72</v>
+      </c>
+      <c r="J5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="6" spans="8:10" x14ac:dyDescent="0.25">
+      <c r="I6" t="s">
+        <v>74</v>
+      </c>
+      <c r="J6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="8:10" x14ac:dyDescent="0.25">
+      <c r="I7" t="s">
+        <v>76</v>
+      </c>
+      <c r="J7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="8:10" x14ac:dyDescent="0.25">
+      <c r="I8" t="s">
+        <v>77</v>
+      </c>
+      <c r="J8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="8:10" x14ac:dyDescent="0.25">
+      <c r="I9" t="s">
+        <v>78</v>
+      </c>
+      <c r="J9">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="8:10" x14ac:dyDescent="0.25">
+      <c r="I10" t="s">
+        <v>79</v>
+      </c>
+      <c r="J10">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="8:10" x14ac:dyDescent="0.25">
+      <c r="I11" t="s">
+        <v>80</v>
+      </c>
+      <c r="J11">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="I2:L19"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="11" max="11" width="25.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="9:12" x14ac:dyDescent="0.25">
+      <c r="L2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="3" spans="9:12" x14ac:dyDescent="0.25">
+      <c r="I3" t="s">
+        <v>84</v>
+      </c>
+      <c r="L3" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="4" spans="9:12" x14ac:dyDescent="0.25">
+      <c r="I4" t="s">
+        <v>87</v>
+      </c>
+      <c r="J4" t="s">
+        <v>86</v>
+      </c>
+      <c r="K4" t="s">
+        <v>72</v>
+      </c>
+      <c r="L4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="5" spans="9:12" x14ac:dyDescent="0.25">
+      <c r="K5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="6" spans="9:12" x14ac:dyDescent="0.25">
+      <c r="K6" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="7" spans="9:12" x14ac:dyDescent="0.25">
+      <c r="K7" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="8" spans="9:12" x14ac:dyDescent="0.25">
+      <c r="K8" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="9" spans="9:12" x14ac:dyDescent="0.25">
+      <c r="K9" s="6" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="10" spans="9:12" x14ac:dyDescent="0.25">
+      <c r="K10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="11" spans="9:12" x14ac:dyDescent="0.25">
+      <c r="K11" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="12" spans="9:12" x14ac:dyDescent="0.25">
+      <c r="K12" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13" spans="9:12" x14ac:dyDescent="0.25">
+      <c r="K13" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="14" spans="9:12" x14ac:dyDescent="0.25">
+      <c r="K14" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="15" spans="9:12" x14ac:dyDescent="0.25">
+      <c r="K15" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="16" spans="9:12" x14ac:dyDescent="0.25">
+      <c r="K16" s="6" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="17" spans="11:11" x14ac:dyDescent="0.25">
+      <c r="K17" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="18" spans="11:11" x14ac:dyDescent="0.25">
+      <c r="K18" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="19" spans="11:11" x14ac:dyDescent="0.25">
+      <c r="K19" s="6" t="s">
+        <v>96</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B2:K11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="5" max="5" width="11.42578125" customWidth="1"/>
+    <col min="6" max="6" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" customWidth="1"/>
+    <col min="10" max="10" width="17.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="K2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="3" spans="2:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="7"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="K3" s="7" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="4" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="J4" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="J5" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="J6" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="J7" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="J8" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="J9" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="J10" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="J11" t="s">
+        <v>117</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="D2:F10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="5" max="5" width="65.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="F2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="3" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D3" t="s">
+        <v>119</v>
+      </c>
+      <c r="E3" t="s">
+        <v>72</v>
+      </c>
+      <c r="F3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="4" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="E4" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="5" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="E5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="E6" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="7" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="E7" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="8" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="E8" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="9" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="E9" s="6" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="10" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="E10" t="s">
+        <v>80</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>